<commit_message>
Complete production level transfer project,And backup of the code before builfig bulkimport of Employee
</commit_message>
<xml_diff>
--- a/Exel formate/Employee_Bulk_Import_.xlsx
+++ b/Exel formate/Employee_Bulk_Import_.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Java\montforterp\ERP-Java\Exel formate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A589EDA-7BCE-4A52-93FB-9EB85480B622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C43E6BE-E9B7-4F0A-A0D0-519005A9CDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
@@ -1230,6 +1230,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="6" width="15.21875" customWidth="1"/>
+    <col min="7" max="7" width="14.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>